<commit_message>
Assign drawing 6 to VW Polo V; add pending drawings 7-12 to registry
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9zuNWHVAw4QsHcaJhMbSm
</commit_message>
<xml_diff>
--- a/specs/Summary_all_drawings.xlsx
+++ b/specs/Summary_all_drawings.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все замечания" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Реестр'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Реестр'!$A$1:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Потребность по моделям'!$A$1:$K$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Каталог'!$A$1:$H$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Все разъёмы'!$A$1:$M$64</definedName>
@@ -478,14 +478,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,6 +515,11 @@
           <t>Папка</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -537,6 +543,11 @@
           <t>specs/Wiring_1</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>готово</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -560,6 +571,11 @@
           <t>specs/Wiring_2</t>
         </is>
       </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>готово</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -583,6 +599,11 @@
           <t>specs/Wiring_3</t>
         </is>
       </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>готово</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -606,6 +627,11 @@
           <t>specs/Wiring_4</t>
         </is>
       </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>готово</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -629,6 +655,11 @@
           <t>specs/Wiring_5</t>
         </is>
       </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>готово</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -636,12 +667,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Volkswagen</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>не указана</t>
+          <t>Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -652,9 +683,146 @@
           <t>specs/Wiring_6</t>
         </is>
       </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>готово</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Niva</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>ожидает схему</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Lada</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Granta Universal</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>ожидает схему</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Lada</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Largus 2012-2021</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>ожидает схему</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Lada</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Largus 2021-</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>ожидает схему</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Lada</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Legend 1993-2021</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>ожидает схему</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Lada</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Niva Travel 2021 Luxe</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>ожидает схему</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -729,7 +897,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>№6 не указана</t>
+          <t>№6 Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -6589,7 +6757,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -6648,7 +6816,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -6707,7 +6875,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -6764,7 +6932,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -6821,7 +6989,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -6880,7 +7048,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -6935,7 +7103,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -6994,7 +7162,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -7053,7 +7221,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -7112,7 +7280,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -7169,7 +7337,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -18977,7 +19145,7 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
@@ -19031,7 +19199,7 @@
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
@@ -19085,7 +19253,7 @@
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
@@ -19139,7 +19307,7 @@
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
@@ -19193,7 +19361,7 @@
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
@@ -19247,7 +19415,7 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
@@ -19301,7 +19469,7 @@
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
@@ -19357,7 +19525,7 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
@@ -19411,7 +19579,7 @@
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
@@ -19465,7 +19633,7 @@
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
@@ -19519,7 +19687,7 @@
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
@@ -19573,7 +19741,7 @@
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
@@ -19627,7 +19795,7 @@
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
@@ -19681,7 +19849,7 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
@@ -19735,7 +19903,7 @@
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
@@ -19789,7 +19957,7 @@
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
@@ -19843,7 +20011,7 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
@@ -19903,7 +20071,7 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
@@ -19963,7 +20131,7 @@
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
@@ -20019,7 +20187,7 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
@@ -20075,7 +20243,7 @@
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
@@ -20133,7 +20301,7 @@
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C230" s="4" t="inlineStr">
@@ -20191,7 +20359,7 @@
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
@@ -20249,7 +20417,7 @@
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
@@ -20307,7 +20475,7 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
@@ -20363,7 +20531,7 @@
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C234" s="4" t="inlineStr">
@@ -20421,7 +20589,7 @@
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr">
@@ -20479,7 +20647,7 @@
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C236" s="4" t="inlineStr">
@@ -20537,7 +20705,7 @@
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C237" s="4" t="inlineStr">
@@ -20595,7 +20763,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -20651,7 +20819,7 @@
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
@@ -20705,7 +20873,7 @@
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
@@ -20759,7 +20927,7 @@
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
@@ -20813,7 +20981,7 @@
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
@@ -20867,7 +21035,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -20921,7 +21089,7 @@
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
@@ -20975,7 +21143,7 @@
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C245" s="4" t="inlineStr">
@@ -21033,7 +21201,7 @@
       </c>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C246" s="4" t="inlineStr">
@@ -21091,7 +21259,7 @@
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
@@ -21145,7 +21313,7 @@
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
@@ -21199,7 +21367,7 @@
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
@@ -21257,7 +21425,7 @@
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C250" s="4" t="inlineStr">
@@ -21315,7 +21483,7 @@
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
@@ -21369,7 +21537,7 @@
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
@@ -21423,7 +21591,7 @@
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
@@ -21477,7 +21645,7 @@
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
@@ -21531,7 +21699,7 @@
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
@@ -21585,7 +21753,7 @@
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
@@ -21641,7 +21809,7 @@
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
@@ -21697,7 +21865,7 @@
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
@@ -21753,7 +21921,7 @@
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
@@ -21809,7 +21977,7 @@
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
@@ -21865,7 +22033,7 @@
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
@@ -21921,7 +22089,7 @@
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
@@ -21977,7 +22145,7 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
@@ -23544,7 +23712,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -23565,7 +23733,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -23586,7 +23754,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -23607,7 +23775,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -23628,7 +23796,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -23649,7 +23817,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -23670,7 +23838,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -23691,7 +23859,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -23712,7 +23880,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -23733,7 +23901,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -23754,7 +23922,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -23775,7 +23943,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -23796,7 +23964,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -23821,7 +23989,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -23846,7 +24014,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -23871,7 +24039,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -23896,7 +24064,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>модель не указана</t>
+          <t>Volkswagen Polo V SD 2010-2020 (1)</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">

</xml_diff>